<commit_message>
chore: update test paths to point to new staging PDP and Blog templates
</commit_message>
<xml_diff>
--- a/docs/GlobeWest_Remediation_Log_Latest.xlsx
+++ b/docs/GlobeWest_Remediation_Log_Latest.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Remediation Log" sheetId="1" r:id="rId1"/>
+    <sheet name="09-07-2026" sheetId="1" r:id="rId1"/>
   </sheets>
 </workbook>
 </file>
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G41"/>
+  <dimension ref="A1:G43"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="25.83203125" customWidth="1"/>
@@ -1351,9 +1351,55 @@
         <v>VERIFIED FIXED</v>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>GW-A11Y-41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>2. PLP (Furniture)</v>
+      </c>
+      <c r="C42" t="str">
+        <v>2.4.4 Link Purpose</v>
+      </c>
+      <c r="D42" t="str">
+        <v>button-name</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Wishlist icon buttons on product grid cards lack accessible text labels.</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Add an aria-label containing the product name to the wishlist button element.</v>
+      </c>
+      <c r="G42" t="str">
+        <v>PENDING REMEDIATION</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>GW-A11Y-42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>2. PLP (Furniture)</v>
+      </c>
+      <c r="C43" t="str">
+        <v>4.1.2 Name Role Value</v>
+      </c>
+      <c r="D43" t="str">
+        <v>nested-interactive</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Sort By selection wrapper element nests interactive select inputs inside a button-role container.</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Remove button role from the select2 container or restructure to prevent nested controls.</v>
+      </c>
+      <c r="G43" t="str">
+        <v>PENDING REMEDIATION</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G41"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G43"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>